<commit_message>
Acrescentado tabela comprovando a maior amostragem nos veículos que possuem um maior km
</commit_message>
<xml_diff>
--- a/Analise_Graficos.xlsx
+++ b/Analise_Graficos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rafae\OneDrive\Documentos\João Oliveira\Portfolio\Preço_dos_Carros\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61FFB78D-5134-4291-A754-46D3BC00D650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54D93087-898F-4054-AB80-12ED774F6631}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Trad" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1383" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1389" uniqueCount="130">
   <si>
     <t>ID Carro</t>
   </si>
@@ -436,6 +436,12 @@
   <si>
     <t>Média de Valor dos Carros</t>
   </si>
+  <si>
+    <t>Preco Medio</t>
+  </si>
+  <si>
+    <t>QTD</t>
+  </si>
 </sst>
 </file>
 
@@ -445,7 +451,7 @@
     <numFmt numFmtId="8" formatCode="&quot;R$&quot;\ #,##0.00;[Red]\-&quot;R$&quot;\ #,##0.00"/>
     <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -461,8 +467,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -473,6 +486,12 @@
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -556,7 +575,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
@@ -574,6 +593,15 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="44" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5943,6 +5971,9 @@
       <c:pivotFmt>
         <c:idx val="1"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -5999,6 +6030,9 @@
       <c:pivotFmt>
         <c:idx val="2"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -6055,6 +6089,9 @@
       <c:pivotFmt>
         <c:idx val="3"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -6111,6 +6148,9 @@
       <c:pivotFmt>
         <c:idx val="4"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -6167,6 +6207,9 @@
       <c:pivotFmt>
         <c:idx val="5"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -6279,6 +6322,9 @@
       <c:pivotFmt>
         <c:idx val="7"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -6335,6 +6381,9 @@
       <c:pivotFmt>
         <c:idx val="8"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -6391,6 +6440,9 @@
       <c:pivotFmt>
         <c:idx val="9"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -6503,6 +6555,9 @@
       <c:pivotFmt>
         <c:idx val="11"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -6559,6 +6614,9 @@
       <c:pivotFmt>
         <c:idx val="12"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -6615,6 +6673,9 @@
       <c:pivotFmt>
         <c:idx val="13"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -6671,6 +6732,9 @@
       <c:pivotFmt>
         <c:idx val="14"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -6727,6 +6791,9 @@
       <c:pivotFmt>
         <c:idx val="15"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -6783,6 +6850,9 @@
       <c:pivotFmt>
         <c:idx val="16"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -6839,6 +6909,9 @@
       <c:pivotFmt>
         <c:idx val="17"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -6895,6 +6968,9 @@
       <c:pivotFmt>
         <c:idx val="18"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -6951,6 +7027,9 @@
       <c:pivotFmt>
         <c:idx val="19"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -7007,6 +7086,9 @@
       <c:pivotFmt>
         <c:idx val="20"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -7063,6 +7145,9 @@
       <c:pivotFmt>
         <c:idx val="21"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -7119,6 +7204,9 @@
       <c:pivotFmt>
         <c:idx val="22"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -7175,6 +7263,9 @@
       <c:pivotFmt>
         <c:idx val="23"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -7231,6 +7322,9 @@
       <c:pivotFmt>
         <c:idx val="24"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -7287,6 +7381,9 @@
       <c:pivotFmt>
         <c:idx val="25"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -7343,6 +7440,9 @@
       <c:pivotFmt>
         <c:idx val="26"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -7399,6 +7499,9 @@
       <c:pivotFmt>
         <c:idx val="27"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -7455,6 +7558,9 @@
       <c:pivotFmt>
         <c:idx val="28"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -7511,6 +7617,9 @@
       <c:pivotFmt>
         <c:idx val="29"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -7567,6 +7676,9 @@
       <c:pivotFmt>
         <c:idx val="30"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -7623,6 +7735,9 @@
       <c:pivotFmt>
         <c:idx val="31"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -7679,6 +7794,9 @@
       <c:pivotFmt>
         <c:idx val="32"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -7735,6 +7853,9 @@
       <c:pivotFmt>
         <c:idx val="33"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -7791,6 +7912,9 @@
       <c:pivotFmt>
         <c:idx val="34"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -7847,6 +7971,9 @@
       <c:pivotFmt>
         <c:idx val="35"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -7903,6 +8030,9 @@
       <c:pivotFmt>
         <c:idx val="36"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -7959,6 +8089,9 @@
       <c:pivotFmt>
         <c:idx val="37"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -8015,6 +8148,9 @@
       <c:pivotFmt>
         <c:idx val="38"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -8071,6 +8207,9 @@
       <c:pivotFmt>
         <c:idx val="39"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -8127,6 +8266,9 @@
       <c:pivotFmt>
         <c:idx val="40"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -8183,6 +8325,9 @@
       <c:pivotFmt>
         <c:idx val="41"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -8239,6 +8384,9 @@
       <c:pivotFmt>
         <c:idx val="42"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -8295,6 +8443,9 @@
       <c:pivotFmt>
         <c:idx val="43"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -8351,6 +8502,9 @@
       <c:pivotFmt>
         <c:idx val="44"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -8407,6 +8561,9 @@
       <c:pivotFmt>
         <c:idx val="45"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -8463,6 +8620,9 @@
       <c:pivotFmt>
         <c:idx val="46"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -8519,6 +8679,9 @@
       <c:pivotFmt>
         <c:idx val="47"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -8575,6 +8738,9 @@
       <c:pivotFmt>
         <c:idx val="48"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -8631,6 +8797,9 @@
       <c:pivotFmt>
         <c:idx val="49"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -8687,6 +8856,9 @@
       <c:pivotFmt>
         <c:idx val="50"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -12776,6 +12948,9 @@
       <c:pivotFmt>
         <c:idx val="54"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -12888,6 +13063,9 @@
       <c:pivotFmt>
         <c:idx val="56"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -12944,6 +13122,9 @@
       <c:pivotFmt>
         <c:idx val="57"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -13000,6 +13181,9 @@
       <c:pivotFmt>
         <c:idx val="58"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -13112,6 +13296,9 @@
       <c:pivotFmt>
         <c:idx val="60"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -13168,6 +13355,9 @@
       <c:pivotFmt>
         <c:idx val="61"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -13224,6 +13414,9 @@
       <c:pivotFmt>
         <c:idx val="62"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -13280,6 +13473,9 @@
       <c:pivotFmt>
         <c:idx val="63"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -13336,6 +13532,9 @@
       <c:pivotFmt>
         <c:idx val="64"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -13392,6 +13591,9 @@
       <c:pivotFmt>
         <c:idx val="65"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -13448,6 +13650,9 @@
       <c:pivotFmt>
         <c:idx val="66"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -13504,6 +13709,9 @@
       <c:pivotFmt>
         <c:idx val="67"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -13560,6 +13768,9 @@
       <c:pivotFmt>
         <c:idx val="68"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -13616,6 +13827,9 @@
       <c:pivotFmt>
         <c:idx val="69"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -13672,6 +13886,9 @@
       <c:pivotFmt>
         <c:idx val="70"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -13728,6 +13945,9 @@
       <c:pivotFmt>
         <c:idx val="71"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -13784,6 +14004,9 @@
       <c:pivotFmt>
         <c:idx val="72"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -13840,6 +14063,9 @@
       <c:pivotFmt>
         <c:idx val="73"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -13896,6 +14122,9 @@
       <c:pivotFmt>
         <c:idx val="74"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -13952,6 +14181,9 @@
       <c:pivotFmt>
         <c:idx val="75"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -14008,6 +14240,9 @@
       <c:pivotFmt>
         <c:idx val="76"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -14064,6 +14299,9 @@
       <c:pivotFmt>
         <c:idx val="77"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -14120,6 +14358,9 @@
       <c:pivotFmt>
         <c:idx val="78"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -14176,6 +14417,9 @@
       <c:pivotFmt>
         <c:idx val="79"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -14232,6 +14476,9 @@
       <c:pivotFmt>
         <c:idx val="80"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -14288,6 +14535,9 @@
       <c:pivotFmt>
         <c:idx val="81"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -14344,6 +14594,9 @@
       <c:pivotFmt>
         <c:idx val="82"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -14400,6 +14653,9 @@
       <c:pivotFmt>
         <c:idx val="83"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -14456,6 +14712,9 @@
       <c:pivotFmt>
         <c:idx val="84"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -14512,6 +14771,9 @@
       <c:pivotFmt>
         <c:idx val="85"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -14568,6 +14830,9 @@
       <c:pivotFmt>
         <c:idx val="86"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -14624,6 +14889,9 @@
       <c:pivotFmt>
         <c:idx val="87"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -14680,6 +14948,9 @@
       <c:pivotFmt>
         <c:idx val="88"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -14736,6 +15007,9 @@
       <c:pivotFmt>
         <c:idx val="89"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -14792,6 +15066,9 @@
       <c:pivotFmt>
         <c:idx val="90"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -14848,6 +15125,9 @@
       <c:pivotFmt>
         <c:idx val="91"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -14904,6 +15184,9 @@
       <c:pivotFmt>
         <c:idx val="92"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -14960,6 +15243,9 @@
       <c:pivotFmt>
         <c:idx val="93"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -15016,6 +15302,9 @@
       <c:pivotFmt>
         <c:idx val="94"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -15072,6 +15361,9 @@
       <c:pivotFmt>
         <c:idx val="95"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -15128,6 +15420,9 @@
       <c:pivotFmt>
         <c:idx val="96"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -15184,6 +15479,9 @@
       <c:pivotFmt>
         <c:idx val="97"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -15240,6 +15538,9 @@
       <c:pivotFmt>
         <c:idx val="98"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -15296,6 +15597,9 @@
       <c:pivotFmt>
         <c:idx val="99"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -15352,6 +15656,9 @@
       <c:pivotFmt>
         <c:idx val="100"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -15408,6 +15715,9 @@
       <c:pivotFmt>
         <c:idx val="101"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -15464,6 +15774,9 @@
       <c:pivotFmt>
         <c:idx val="102"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -15520,6 +15833,9 @@
       <c:pivotFmt>
         <c:idx val="103"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -32636,7 +32952,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{109E1C2A-721A-4280-B812-D51065658051}">
-  <dimension ref="A3:E7"/>
+  <dimension ref="A3:E32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.5703125" bestFit="1" customWidth="1"/>
@@ -32718,6 +33034,50 @@
       </c>
       <c r="E7" s="5">
         <v>52629.885000000002</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="B30" s="15">
+        <v>52785.91</v>
+      </c>
+      <c r="C30" s="14">
+        <v>1986</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="B31" s="15">
+        <v>52249.42</v>
+      </c>
+      <c r="C31" s="14">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B32" s="15">
+        <v>51738.71</v>
+      </c>
+      <c r="C32" s="14">
+        <v>184</v>
       </c>
     </row>
   </sheetData>

</xml_diff>